<commit_message>
Book bonus provision into Grouped Trial Balance (restated)
- New expense GL X2001002003010 Bonus (8.33% on Basic+DA, eligible <=21k/mo) Dr 20,492,342.50 under Employee Benefit Expense
- Bonus Payable (L2007002003001) Cr 20,492,342.50
- Summary by Head: EBE Dr 20,688,580.50; Employee Payables Cr 20,492,342.50
- Grand total 634,933,159.91 (Dr=Cr), TB ties
</commit_message>
<xml_diff>
--- a/docs/maharashtra/Maharashtra_Trial_Balance_GROUPED_Dep_per_Schedule_FY24-25.xlsx
+++ b/docs/maharashtra/Maharashtra_Trial_Balance_GROUPED_Dep_per_Schedule_FY24-25.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -512,6 +512,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2172,7 +2173,9 @@
         </is>
       </c>
       <c r="C70" s="5" t="n"/>
-      <c r="D70" s="5" t="n"/>
+      <c r="D70" s="5" t="n">
+        <v>20492342.5</v>
+      </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
           <t>Employee related payables</t>
@@ -3117,42 +3120,42 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>X2001003004001</t>
+          <t>X2001002003010</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>INTERNET EXPENSE-18%</t>
+          <t>BONUS (PROVISION @ 8.33% ON BASIC+DA, ELIGIBLE &lt;= Rs.21,000/MO)</t>
         </is>
       </c>
       <c r="C107" s="5" t="n">
-        <v>37384.52</v>
+        <v>20492342.5</v>
       </c>
       <c r="D107" s="5" t="n"/>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>Communication Expenses</t>
+          <t>Employee benefit expenses</t>
         </is>
       </c>
       <c r="F107" s="4" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Employee Benefit Expense</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>X2001003004002</t>
+          <t>X2001003004001</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>MOBILE EXPENSE-18%</t>
+          <t>INTERNET EXPENSE-18%</t>
         </is>
       </c>
       <c r="C108" s="5" t="n">
-        <v>55023.5</v>
+        <v>37384.52</v>
       </c>
       <c r="D108" s="5" t="n"/>
       <c r="E108" s="4" t="inlineStr">
@@ -3169,16 +3172,16 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>X2001003004004</t>
+          <t>X2001003004002</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>POSTAGE &amp; COURIER EXPENSE</t>
+          <t>MOBILE EXPENSE-18%</t>
         </is>
       </c>
       <c r="C109" s="5" t="n">
-        <v>76567</v>
+        <v>55023.5</v>
       </c>
       <c r="D109" s="5" t="n"/>
       <c r="E109" s="4" t="inlineStr">
@@ -3195,16 +3198,16 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>X2001003004006</t>
+          <t>X2001003004004</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>INTERNET EXPENSE</t>
+          <t>POSTAGE &amp; COURIER EXPENSE</t>
         </is>
       </c>
       <c r="C110" s="5" t="n">
-        <v>10</v>
+        <v>76567</v>
       </c>
       <c r="D110" s="5" t="n"/>
       <c r="E110" s="4" t="inlineStr">
@@ -3221,21 +3224,21 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>X2001003005001</t>
+          <t>X2001003004006</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>CONVEYANCE EXPENSE</t>
+          <t>INTERNET EXPENSE</t>
         </is>
       </c>
       <c r="C111" s="5" t="n">
-        <v>17874</v>
+        <v>10</v>
       </c>
       <c r="D111" s="5" t="n"/>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>Travelling &amp; Conveyance</t>
+          <t>Communication Expenses</t>
         </is>
       </c>
       <c r="F111" s="4" t="inlineStr">
@@ -3247,16 +3250,16 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>X2001003005002</t>
+          <t>X2001003005001</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>TOUR &amp; TRAVELLING EXPENSE</t>
+          <t>CONVEYANCE EXPENSE</t>
         </is>
       </c>
       <c r="C112" s="5" t="n">
-        <v>103534.08</v>
+        <v>17874</v>
       </c>
       <c r="D112" s="5" t="n"/>
       <c r="E112" s="4" t="inlineStr">
@@ -3273,16 +3276,16 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>X2001003005005</t>
+          <t>X2001003005002</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>PETROL OIL &amp; FUEL EXPENSE</t>
+          <t>TOUR &amp; TRAVELLING EXPENSE</t>
         </is>
       </c>
       <c r="C113" s="5" t="n">
-        <v>500</v>
+        <v>103534.08</v>
       </c>
       <c r="D113" s="5" t="n"/>
       <c r="E113" s="4" t="inlineStr">
@@ -3299,16 +3302,16 @@
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>X2001003005007</t>
+          <t>X2001003005005</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>TOUR &amp; TRAVELLING EXPENSE-5%</t>
+          <t>PETROL OIL &amp; FUEL EXPENSE</t>
         </is>
       </c>
       <c r="C114" s="5" t="n">
-        <v>6922</v>
+        <v>500</v>
       </c>
       <c r="D114" s="5" t="n"/>
       <c r="E114" s="4" t="inlineStr">
@@ -3325,21 +3328,21 @@
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>X2001003006002</t>
+          <t>X2001003005007</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>ELECTRICITY EXPENSE</t>
+          <t>TOUR &amp; TRAVELLING EXPENSE-5%</t>
         </is>
       </c>
       <c r="C115" s="5" t="n">
-        <v>263240</v>
+        <v>6922</v>
       </c>
       <c r="D115" s="5" t="n"/>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>Electricity &amp; Water</t>
+          <t>Travelling &amp; Conveyance</t>
         </is>
       </c>
       <c r="F115" s="4" t="inlineStr">
@@ -3351,21 +3354,21 @@
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>X2001003010002</t>
+          <t>X2001003006002</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>PROFESSIONAL &amp; CONSULTANCY CHARGE-18%</t>
+          <t>ELECTRICITY EXPENSE</t>
         </is>
       </c>
       <c r="C116" s="5" t="n">
-        <v>100000</v>
+        <v>263240</v>
       </c>
       <c r="D116" s="5" t="n"/>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Charges</t>
+          <t>Electricity &amp; Water</t>
         </is>
       </c>
       <c r="F116" s="4" t="inlineStr">
@@ -3377,21 +3380,21 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>X2001003011002005</t>
+          <t>X2001003010002</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>SUBSCRIPTION &amp; MEMBERSHIP FEE 18%</t>
+          <t>PROFESSIONAL &amp; CONSULTANCY CHARGE-18%</t>
         </is>
       </c>
       <c r="C117" s="5" t="n">
-        <v>764</v>
+        <v>100000</v>
       </c>
       <c r="D117" s="5" t="n"/>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>Fees &amp; Taxes</t>
+          <t>Legal &amp; Professional Charges</t>
         </is>
       </c>
       <c r="F117" s="4" t="inlineStr">
@@ -3403,68 +3406,68 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>X2001003011002007</t>
+          <t>X2001003011002005</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>GST INTEREST</t>
+          <t>SUBSCRIPTION &amp; MEMBERSHIP FEE 18%</t>
         </is>
       </c>
       <c r="C118" s="5" t="n">
-        <v>2451</v>
+        <v>764</v>
       </c>
       <c r="D118" s="5" t="n"/>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>Other Interest</t>
+          <t>Fees &amp; Taxes</t>
         </is>
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>Finance Costs</t>
+          <t>Other Expenses</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>X2001003011002009</t>
+          <t>X2001003011002007</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>FEES &amp; TAXES</t>
+          <t>GST INTEREST</t>
         </is>
       </c>
       <c r="C119" s="5" t="n">
-        <v>118</v>
+        <v>2451</v>
       </c>
       <c r="D119" s="5" t="n"/>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>Fees &amp; Taxes</t>
+          <t>Other Interest</t>
         </is>
       </c>
       <c r="F119" s="4" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Finance Costs</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>X2001003011002011</t>
+          <t>X2001003011002009</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>LATE FEE-GST</t>
+          <t>FEES &amp; TAXES</t>
         </is>
       </c>
       <c r="C120" s="5" t="n">
-        <v>102850</v>
+        <v>118</v>
       </c>
       <c r="D120" s="5" t="n"/>
       <c r="E120" s="4" t="inlineStr">
@@ -3481,21 +3484,21 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>X2001003011004003</t>
+          <t>X2001003011002011</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>FOODING DEDUCTION</t>
+          <t>LATE FEE-GST</t>
         </is>
       </c>
       <c r="C121" s="5" t="n">
-        <v>66193</v>
+        <v>102850</v>
       </c>
       <c r="D121" s="5" t="n"/>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>Fooding deduction</t>
+          <t>Fees &amp; Taxes</t>
         </is>
       </c>
       <c r="F121" s="4" t="inlineStr">
@@ -3507,21 +3510,21 @@
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>X2001003011004004</t>
+          <t>X2001003011004003</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>OTHER DEDUCTION.</t>
+          <t>FOODING DEDUCTION</t>
         </is>
       </c>
       <c r="C122" s="5" t="n">
-        <v>12741.63</v>
+        <v>66193</v>
       </c>
       <c r="D122" s="5" t="n"/>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>other deduction</t>
+          <t>Fooding deduction</t>
         </is>
       </c>
       <c r="F122" s="4" t="inlineStr">
@@ -3533,21 +3536,21 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005007</t>
+          <t>X2001003011004004</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>POSTAGE &amp; COURIER EXPENSES-18%</t>
+          <t>OTHER DEDUCTION.</t>
         </is>
       </c>
       <c r="C123" s="5" t="n">
-        <v>6840</v>
+        <v>12741.63</v>
       </c>
       <c r="D123" s="5" t="n"/>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>Communication Expenses</t>
+          <t>other deduction</t>
         </is>
       </c>
       <c r="F123" s="4" t="inlineStr">
@@ -3559,21 +3562,21 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005013</t>
+          <t>X2001003011005007</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>LOW VALUE ASSET EXPENSE-18%</t>
+          <t>POSTAGE &amp; COURIER EXPENSES-18%</t>
         </is>
       </c>
       <c r="C124" s="5" t="n">
-        <v>3387.29</v>
+        <v>6840</v>
       </c>
       <c r="D124" s="5" t="n"/>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>Misscellaneous Expenses</t>
+          <t>Communication Expenses</t>
         </is>
       </c>
       <c r="F124" s="4" t="inlineStr">
@@ -3585,16 +3588,16 @@
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005014</t>
+          <t>X2001003011005013</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>POLICE VERIFICATION EXPENSE</t>
+          <t>LOW VALUE ASSET EXPENSE-18%</t>
         </is>
       </c>
       <c r="C125" s="5" t="n">
-        <v>95200</v>
+        <v>3387.29</v>
       </c>
       <c r="D125" s="5" t="n"/>
       <c r="E125" s="4" t="inlineStr">
@@ -3611,18 +3614,18 @@
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005015</t>
+          <t>X2001003011005014</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>ROUND OFF.</t>
-        </is>
-      </c>
-      <c r="C126" s="5" t="n"/>
-      <c r="D126" s="5" t="n">
-        <v>1000.89</v>
-      </c>
+          <t>POLICE VERIFICATION EXPENSE</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="n">
+        <v>95200</v>
+      </c>
+      <c r="D126" s="5" t="n"/>
       <c r="E126" s="4" t="inlineStr">
         <is>
           <t>Misscellaneous Expenses</t>
@@ -3637,18 +3640,18 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005017</t>
+          <t>X2001003011005015</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>OTHER OFFICE EXPENSE</t>
-        </is>
-      </c>
-      <c r="C127" s="5" t="n">
-        <v>1100</v>
-      </c>
-      <c r="D127" s="5" t="n"/>
+          <t>ROUND OFF.</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="n"/>
+      <c r="D127" s="5" t="n">
+        <v>1000.89</v>
+      </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
           <t>Misscellaneous Expenses</t>
@@ -3663,16 +3666,16 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005018</t>
+          <t>X2001003011005017</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>SHORT &amp; EXCESS</t>
+          <t>OTHER OFFICE EXPENSE</t>
         </is>
       </c>
       <c r="C128" s="5" t="n">
-        <v>58.84</v>
+        <v>1100</v>
       </c>
       <c r="D128" s="5" t="n"/>
       <c r="E128" s="4" t="inlineStr">
@@ -3689,16 +3692,16 @@
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005024</t>
+          <t>X2001003011005018</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>DISCOUNT &amp; AMT W/OFF</t>
+          <t>SHORT &amp; EXCESS</t>
         </is>
       </c>
       <c r="C129" s="5" t="n">
-        <v>140806.95</v>
+        <v>58.84</v>
       </c>
       <c r="D129" s="5" t="n"/>
       <c r="E129" s="4" t="inlineStr">
@@ -3715,73 +3718,73 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005027</t>
+          <t>X2001003011005024</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>SITE EXPENSE OTHER</t>
+          <t>DISCOUNT &amp; AMT W/OFF</t>
         </is>
       </c>
       <c r="C130" s="5" t="n">
-        <v>7050</v>
+        <v>140806.95</v>
       </c>
       <c r="D130" s="5" t="n"/>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>Site Expense</t>
+          <t>Misscellaneous Expenses</t>
         </is>
       </c>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>Direct Site Expenses (Cost of Services)</t>
+          <t>Other Expenses</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>X2001003011005028</t>
+          <t>X2001003011005027</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>LOW VALUE ASSET EXPENSE</t>
+          <t>SITE EXPENSE OTHER</t>
         </is>
       </c>
       <c r="C131" s="5" t="n">
-        <v>800</v>
+        <v>7050</v>
       </c>
       <c r="D131" s="5" t="n"/>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>Misscellaneous Expenses</t>
+          <t>Site Expense</t>
         </is>
       </c>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Direct Site Expenses (Cost of Services)</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>X2001003011006001</t>
+          <t>X2001003011005028</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>FESTIVAL EXPENSE</t>
+          <t>LOW VALUE ASSET EXPENSE</t>
         </is>
       </c>
       <c r="C132" s="5" t="n">
-        <v>51000</v>
+        <v>800</v>
       </c>
       <c r="D132" s="5" t="n"/>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>Diwali Expenses</t>
+          <t>Misscellaneous Expenses</t>
         </is>
       </c>
       <c r="F132" s="4" t="inlineStr">
@@ -3793,21 +3796,21 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>X2001003012001</t>
+          <t>X2001003011006001</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>PHOTOCOPY &amp; FAX EXPENSE-18%</t>
+          <t>FESTIVAL EXPENSE</t>
         </is>
       </c>
       <c r="C133" s="5" t="n">
-        <v>82800</v>
+        <v>51000</v>
       </c>
       <c r="D133" s="5" t="n"/>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>Printing &amp; Stationery</t>
+          <t>Diwali Expenses</t>
         </is>
       </c>
       <c r="F133" s="4" t="inlineStr">
@@ -3819,16 +3822,16 @@
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>X2001003012004</t>
+          <t>X2001003012001</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>PHOTOCOPY &amp; FAX EXPENSE</t>
+          <t>PHOTOCOPY &amp; FAX EXPENSE-18%</t>
         </is>
       </c>
       <c r="C134" s="5" t="n">
-        <v>1100</v>
+        <v>82800</v>
       </c>
       <c r="D134" s="5" t="n"/>
       <c r="E134" s="4" t="inlineStr">
@@ -3845,16 +3848,16 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>X2001003012005</t>
+          <t>X2001003012004</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>PRINTING &amp; STATIONERY EXPENSE-12%</t>
+          <t>PHOTOCOPY &amp; FAX EXPENSE</t>
         </is>
       </c>
       <c r="C135" s="5" t="n">
-        <v>52662</v>
+        <v>1100</v>
       </c>
       <c r="D135" s="5" t="n"/>
       <c r="E135" s="4" t="inlineStr">
@@ -3871,16 +3874,16 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>X2001003012006</t>
+          <t>X2001003012005</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>PRINTING &amp; STATIONERY EXPENSE-18%</t>
+          <t>PRINTING &amp; STATIONERY EXPENSE-12%</t>
         </is>
       </c>
       <c r="C136" s="5" t="n">
-        <v>29346</v>
+        <v>52662</v>
       </c>
       <c r="D136" s="5" t="n"/>
       <c r="E136" s="4" t="inlineStr">
@@ -3897,16 +3900,16 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>X2001003012007</t>
+          <t>X2001003012006</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>PRINTING &amp; STATIONERY EXPENSE-SITE</t>
+          <t>PRINTING &amp; STATIONERY EXPENSE-18%</t>
         </is>
       </c>
       <c r="C137" s="5" t="n">
-        <v>6691</v>
+        <v>29346</v>
       </c>
       <c r="D137" s="5" t="n"/>
       <c r="E137" s="4" t="inlineStr">
@@ -3923,21 +3926,21 @@
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>X2001003014001001</t>
+          <t>X2001003012007</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>REPAIR &amp; MAINTENANCE-MACHINERY.</t>
+          <t>PRINTING &amp; STATIONERY EXPENSE-SITE</t>
         </is>
       </c>
       <c r="C138" s="5" t="n">
-        <v>38638</v>
+        <v>6691</v>
       </c>
       <c r="D138" s="5" t="n"/>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>Repair and Maintenance-machinery</t>
+          <t>Printing &amp; Stationery</t>
         </is>
       </c>
       <c r="F138" s="4" t="inlineStr">
@@ -3949,16 +3952,16 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>X2001003014001002</t>
+          <t>X2001003014001001</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>REPAIR &amp; MAINTENANCE EXPENSE MACHINERY-18%</t>
+          <t>REPAIR &amp; MAINTENANCE-MACHINERY.</t>
         </is>
       </c>
       <c r="C139" s="5" t="n">
-        <v>4450</v>
+        <v>38638</v>
       </c>
       <c r="D139" s="5" t="n"/>
       <c r="E139" s="4" t="inlineStr">
@@ -3975,21 +3978,21 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>X2001003014002004</t>
+          <t>X2001003014001002</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>REPAIR &amp; MAINTENANCE EXPENSE-OTHERS</t>
+          <t>REPAIR &amp; MAINTENANCE EXPENSE MACHINERY-18%</t>
         </is>
       </c>
       <c r="C140" s="5" t="n">
-        <v>8770</v>
+        <v>4450</v>
       </c>
       <c r="D140" s="5" t="n"/>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>Others Repairs</t>
+          <t>Repair and Maintenance-machinery</t>
         </is>
       </c>
       <c r="F140" s="4" t="inlineStr">
@@ -4001,16 +4004,16 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>X2001003014002013</t>
+          <t>X2001003014002004</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>REPAIR &amp; MAINTENANCE EXPENSE-COMPUTER</t>
+          <t>REPAIR &amp; MAINTENANCE EXPENSE-OTHERS</t>
         </is>
       </c>
       <c r="C141" s="5" t="n">
-        <v>2038</v>
+        <v>8770</v>
       </c>
       <c r="D141" s="5" t="n"/>
       <c r="E141" s="4" t="inlineStr">
@@ -4027,16 +4030,16 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>X2001003014002015</t>
+          <t>X2001003014002013</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>REPAIR &amp; MAINTENANCE EXPENSE-ELECTRIC</t>
+          <t>REPAIR &amp; MAINTENANCE EXPENSE-COMPUTER</t>
         </is>
       </c>
       <c r="C142" s="5" t="n">
-        <v>430</v>
+        <v>2038</v>
       </c>
       <c r="D142" s="5" t="n"/>
       <c r="E142" s="4" t="inlineStr">
@@ -4053,96 +4056,122 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>X2001003016001</t>
+          <t>X2001003014002015</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>RENT-18%</t>
+          <t>REPAIR &amp; MAINTENANCE EXPENSE-ELECTRIC</t>
         </is>
       </c>
       <c r="C143" s="5" t="n">
-        <v>354000</v>
+        <v>430</v>
       </c>
       <c r="D143" s="5" t="n"/>
       <c r="E143" s="4" t="inlineStr">
         <is>
+          <t>Others Repairs</t>
+        </is>
+      </c>
+      <c r="F143" s="4" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="inlineStr">
+        <is>
+          <t>X2001003016001</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>RENT-18%</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="n">
+        <v>354000</v>
+      </c>
+      <c r="D144" s="5" t="n"/>
+      <c r="E144" s="4" t="inlineStr">
+        <is>
           <t>Rent</t>
         </is>
       </c>
-      <c r="F143" s="4" t="inlineStr">
+      <c r="F144" s="4" t="inlineStr">
         <is>
           <t>Other Expenses</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t>DEP-001</t>
-        </is>
-      </c>
-      <c r="B144" s="6" t="inlineStr">
-        <is>
-          <t>DEPRECIATION FOR THE YEAR (as per attached schedule)</t>
-        </is>
-      </c>
-      <c r="C144" s="7" t="n">
-        <v>2604427.71</v>
-      </c>
-      <c r="D144" s="7" t="n"/>
-      <c r="E144" s="6" t="inlineStr">
-        <is>
-          <t>Depreciation</t>
-        </is>
-      </c>
-      <c r="F144" s="6" t="inlineStr">
-        <is>
-          <t>Depreciation</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
+          <t>DEP-001</t>
+        </is>
+      </c>
+      <c r="B145" s="6" t="inlineStr">
+        <is>
+          <t>DEPRECIATION FOR THE YEAR (as per attached schedule)</t>
+        </is>
+      </c>
+      <c r="C145" s="7" t="n">
+        <v>2604427.71</v>
+      </c>
+      <c r="D145" s="7" t="n"/>
+      <c r="E145" s="6" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="F145" s="6" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="inlineStr">
+        <is>
           <t>HO-ADJ</t>
         </is>
       </c>
-      <c r="B145" s="6" t="inlineStr">
+      <c r="B146" s="6" t="inlineStr">
         <is>
           <t>HEAD OFFICE / INTER-UNIT A/C — building (net WDV) brought into branch books + computer dep reversal (contra); incl. TB rounding</t>
         </is>
       </c>
-      <c r="C145" s="7" t="n"/>
-      <c r="D145" s="7" t="n">
+      <c r="C146" s="7" t="n"/>
+      <c r="D146" s="7" t="n">
         <v>13849100.22</v>
       </c>
-      <c r="E145" s="6" t="inlineStr">
+      <c r="E146" s="6" t="inlineStr">
         <is>
           <t>INTERUNIT</t>
         </is>
       </c>
-      <c r="F145" s="6" t="inlineStr">
+      <c r="F146" s="6" t="inlineStr">
         <is>
           <t>Inter-Unit / Branch</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="8" t="n"/>
-      <c r="B146" s="8" t="inlineStr">
+    <row r="147">
+      <c r="A147" s="8" t="n"/>
+      <c r="B147" s="8" t="inlineStr">
         <is>
           <t>GRAND TOTAL (restated)</t>
         </is>
       </c>
-      <c r="C146" s="9" t="n">
-        <v>614440817.41</v>
-      </c>
-      <c r="D146" s="9" t="n">
-        <v>614440817.41</v>
-      </c>
-      <c r="E146" s="8" t="n"/>
-      <c r="F146" s="8" t="n"/>
+      <c r="C147" s="9" t="n">
+        <v>634933159.91</v>
+      </c>
+      <c r="D147" s="9" t="n">
+        <v>634933159.91</v>
+      </c>
+      <c r="E147" s="8" t="n"/>
+      <c r="F147" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4706,6 +4735,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -4930,10 +4960,10 @@
         <v>0</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>0</v>
+        <v>20492342.5</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0</v>
+        <v>-20492342.5</v>
       </c>
     </row>
     <row r="17">
@@ -5023,13 +5053,13 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>196238</v>
+        <v>20688580.5</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>196238</v>
+        <v>20688580.5</v>
       </c>
     </row>
     <row r="23">
@@ -5087,13 +5117,13 @@
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>614440817.41</v>
+        <v>634933159.91</v>
       </c>
       <c r="C26" s="9" t="n">
-        <v>614440817.41</v>
+        <v>634933159.91</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>